<commit_message>
Atualiza análise de desempenho por ano
</commit_message>
<xml_diff>
--- a/backend/data/desempenho_por_ano_analise.xlsx
+++ b/backend/data/desempenho_por_ano_analise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo\Dropbox\Codex\paineldadosavalie2026.2\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED106C2-AABA-4F17-BC32-0AEF76208E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A53D50BD-177C-4A63-A80A-6028BD0EDEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>Classificação</t>
   </si>
   <si>
-    <t>Habilidades Críticas (nº)</t>
-  </si>
-  <si>
     <t>EEF 21 DE DEZEMBRO</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>Base da Rede</t>
+  </si>
+  <si>
+    <t>Habilidades Críticas até 56% (nº)</t>
   </si>
 </sst>
 </file>
@@ -381,6 +381,15 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -392,15 +401,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -710,22 +710,22 @@
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="8" width="16.6640625" customWidth="1"/>
     <col min="9" max="9" width="16.6640625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" customWidth="1"/>
+    <col min="10" max="10" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="20"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="23"/>
     </row>
     <row r="2" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -756,15 +756,15 @@
         <v>9</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>12</v>
       </c>
       <c r="C3" s="7">
         <v>0.79300000000000004</v>
@@ -792,16 +792,16 @@
         <f t="shared" ref="I3:I34" si="4">IF(E3&gt;=70%,"Adequado",IF(E3&gt;=60%,"Regular","Atenção"))</f>
         <v>Adequado</v>
       </c>
-      <c r="J3" s="24">
-        <v>12</v>
+      <c r="J3" s="19">
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="12">
         <v>0.69299999999999995</v>
@@ -829,16 +829,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J4" s="25">
+      <c r="J4" s="20">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="C5" s="7">
         <v>0.72299999999999998</v>
@@ -866,16 +866,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J5" s="24">
-        <v>0</v>
+      <c r="J5" s="19">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" s="12">
         <v>0.83</v>
@@ -903,16 +903,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J6" s="25">
-        <v>1</v>
+      <c r="J6" s="20">
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="7">
         <v>0.80600000000000005</v>
@@ -940,16 +940,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J7" s="24">
-        <v>0</v>
+      <c r="J7" s="19">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" s="12">
         <v>0.64100000000000001</v>
@@ -977,16 +977,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J8" s="25">
-        <v>1</v>
+      <c r="J8" s="20">
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="7">
         <v>0.83799999999999997</v>
@@ -1014,16 +1014,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J9" s="24">
-        <v>7</v>
+      <c r="J9" s="19">
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="12">
         <v>0.70399999999999996</v>
@@ -1051,16 +1051,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="20">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="7">
         <v>0.66700000000000004</v>
@@ -1088,16 +1088,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J11" s="24">
-        <v>12</v>
+      <c r="J11" s="19">
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="12">
         <v>0.67300000000000004</v>
@@ -1125,16 +1125,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="20">
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="7">
         <v>0.78100000000000003</v>
@@ -1162,16 +1162,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J13" s="24">
-        <v>24</v>
+      <c r="J13" s="19">
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" s="12">
         <v>0.69399999999999995</v>
@@ -1199,16 +1199,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J14" s="25">
-        <v>0</v>
+      <c r="J14" s="20">
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" s="7">
         <v>0.69299999999999995</v>
@@ -1236,16 +1236,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J15" s="24">
-        <v>1</v>
+      <c r="J15" s="19">
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C16" s="12">
         <v>0.67200000000000004</v>
@@ -1273,16 +1273,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J16" s="25">
-        <v>0</v>
+      <c r="J16" s="20">
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17" s="7">
         <v>0.60299999999999998</v>
@@ -1310,16 +1310,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J17" s="24">
-        <v>2</v>
+      <c r="J17" s="19">
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C18" s="12">
         <v>0.59</v>
@@ -1347,16 +1347,16 @@
         <f t="shared" si="4"/>
         <v>Atenção</v>
       </c>
-      <c r="J18" s="25">
-        <v>11</v>
+      <c r="J18" s="20">
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" s="7">
         <v>0.78600000000000003</v>
@@ -1384,16 +1384,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="19">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C20" s="12">
         <v>0.83499999999999996</v>
@@ -1421,16 +1421,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J20" s="25">
+      <c r="J20" s="20">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" s="7">
         <v>0.74099999999999999</v>
@@ -1458,16 +1458,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J21" s="24">
+      <c r="J21" s="19">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" s="12">
         <v>0.82399999999999995</v>
@@ -1495,16 +1495,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J22" s="25">
+      <c r="J22" s="20">
         <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="7">
         <v>0.77200000000000002</v>
@@ -1532,16 +1532,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J23" s="24">
-        <v>7</v>
+      <c r="J23" s="19">
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C24" s="12">
         <v>0.79800000000000004</v>
@@ -1569,16 +1569,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J24" s="25">
-        <v>4</v>
+      <c r="J24" s="20">
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C25" s="7">
         <v>0.82799999999999996</v>
@@ -1606,16 +1606,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J25" s="24">
+      <c r="J25" s="19">
         <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C26" s="12">
         <v>0.73599999999999999</v>
@@ -1643,16 +1643,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J26" s="25">
-        <v>13</v>
+      <c r="J26" s="20">
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C27" s="7">
         <v>0.75600000000000001</v>
@@ -1680,16 +1680,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J27" s="24">
+      <c r="J27" s="19">
         <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C28" s="12">
         <v>0.84099999999999997</v>
@@ -1717,16 +1717,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J28" s="25">
-        <v>0</v>
+      <c r="J28" s="20">
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C29" s="7">
         <v>0.79800000000000004</v>
@@ -1754,16 +1754,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J29" s="24">
-        <v>1</v>
+      <c r="J29" s="19">
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C30" s="12">
         <v>0.57599999999999996</v>
@@ -1791,16 +1791,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J30" s="25">
-        <v>0</v>
+      <c r="J30" s="20">
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C31" s="7">
         <v>0.82299999999999995</v>
@@ -1828,16 +1828,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J31" s="24">
-        <v>2</v>
+      <c r="J31" s="19">
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C32" s="12">
         <v>0.56799999999999995</v>
@@ -1865,16 +1865,16 @@
         <f t="shared" si="4"/>
         <v>Regular</v>
       </c>
-      <c r="J32" s="25">
-        <v>7</v>
+      <c r="J32" s="20">
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C33" s="7">
         <v>0.621</v>
@@ -1902,16 +1902,16 @@
         <f t="shared" si="4"/>
         <v>Atenção</v>
       </c>
-      <c r="J33" s="24">
-        <v>10</v>
+      <c r="J33" s="19">
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C34" s="12">
         <v>0.82399999999999995</v>
@@ -1939,16 +1939,16 @@
         <f t="shared" si="4"/>
         <v>Adequado</v>
       </c>
-      <c r="J34" s="25">
-        <v>12</v>
+      <c r="J34" s="20">
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C35" s="7">
         <v>0.60199999999999998</v>
@@ -1957,7 +1957,7 @@
         <v>0.63600000000000001</v>
       </c>
       <c r="E35" s="7">
-        <f t="shared" ref="E35:E66" si="5">ROUND(AVERAGE(C35,D35),3)</f>
+        <f t="shared" ref="E35:E52" si="5">ROUND(AVERAGE(C35,D35),3)</f>
         <v>0.61899999999999999</v>
       </c>
       <c r="F35" s="8">
@@ -1976,16 +1976,16 @@
         <f t="shared" ref="I35:I52" si="9">IF(E35&gt;=70%,"Adequado",IF(E35&gt;=60%,"Regular","Atenção"))</f>
         <v>Regular</v>
       </c>
-      <c r="J35" s="24">
+      <c r="J35" s="19">
         <v>14</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C36" s="12">
         <v>0.66200000000000003</v>
@@ -2013,16 +2013,16 @@
         <f t="shared" si="9"/>
         <v>Regular</v>
       </c>
-      <c r="J36" s="25">
-        <v>2</v>
+      <c r="J36" s="20">
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C37" s="7">
         <v>0.79900000000000004</v>
@@ -2050,16 +2050,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J37" s="24">
-        <v>0</v>
+      <c r="J37" s="19">
+        <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C38" s="12">
         <v>0.82699999999999996</v>
@@ -2087,16 +2087,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J38" s="25">
-        <v>1</v>
+      <c r="J38" s="20">
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C39" s="7">
         <v>0.77</v>
@@ -2124,16 +2124,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J39" s="24">
-        <v>0</v>
+      <c r="J39" s="19">
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C40" s="12">
         <v>0.70299999999999996</v>
@@ -2161,16 +2161,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J40" s="25">
-        <v>2</v>
+      <c r="J40" s="20">
+        <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C41" s="7">
         <v>0.63400000000000001</v>
@@ -2198,16 +2198,16 @@
         <f t="shared" si="9"/>
         <v>Regular</v>
       </c>
-      <c r="J41" s="24">
-        <v>7</v>
+      <c r="J41" s="19">
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C42" s="12">
         <v>0.86</v>
@@ -2235,16 +2235,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J42" s="25">
-        <v>4</v>
+      <c r="J42" s="20">
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C43" s="7">
         <v>0.84699999999999998</v>
@@ -2272,16 +2272,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J43" s="24">
-        <v>12</v>
+      <c r="J43" s="19">
+        <v>15</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C44" s="12">
         <v>0.72799999999999998</v>
@@ -2309,16 +2309,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J44" s="25">
-        <v>14</v>
+      <c r="J44" s="20">
+        <v>15</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C45" s="7">
         <v>0.69799999999999995</v>
@@ -2346,16 +2346,16 @@
         <f t="shared" si="9"/>
         <v>Regular</v>
       </c>
-      <c r="J45" s="24">
-        <v>23</v>
+      <c r="J45" s="19">
+        <v>25</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C46" s="12">
         <v>0.69699999999999995</v>
@@ -2383,16 +2383,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J46" s="25">
-        <v>0</v>
+      <c r="J46" s="20">
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C47" s="7">
         <v>0.68799999999999994</v>
@@ -2420,16 +2420,16 @@
         <f t="shared" si="9"/>
         <v>Regular</v>
       </c>
-      <c r="J47" s="24">
-        <v>1</v>
+      <c r="J47" s="19">
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C48" s="12">
         <v>0.61599999999999999</v>
@@ -2457,16 +2457,16 @@
         <f t="shared" si="9"/>
         <v>Regular</v>
       </c>
-      <c r="J48" s="25">
-        <v>0</v>
+      <c r="J48" s="20">
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C49" s="7">
         <v>0.76500000000000001</v>
@@ -2494,16 +2494,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J49" s="24">
-        <v>2</v>
+      <c r="J49" s="19">
+        <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C50" s="12">
         <v>0.71299999999999997</v>
@@ -2531,16 +2531,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J50" s="25">
-        <v>6</v>
+      <c r="J50" s="20">
+        <v>11</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C51" s="7">
         <v>0.71499999999999997</v>
@@ -2568,16 +2568,16 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J51" s="24">
-        <v>4</v>
+      <c r="J51" s="19">
+        <v>7</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C52" s="12">
         <v>0.84199999999999997</v>
@@ -2605,15 +2605,15 @@
         <f t="shared" si="9"/>
         <v>Adequado</v>
       </c>
-      <c r="J52" s="25">
-        <v>12</v>
+      <c r="J52" s="20">
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A53" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="B53" s="23"/>
+      <c r="A53" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B53" s="26"/>
       <c r="C53" s="15">
         <f>AVERAGE(C3:C52)</f>
         <v>0.7338800000000002</v>
@@ -2631,17 +2631,17 @@
         <v>0.36200000000002897</v>
       </c>
       <c r="G53" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="H53" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="I53" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="H53" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="I53" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="J53" s="26">
+      <c r="J53" s="21">
         <f>AVERAGE(J3:J52)</f>
-        <v>6.28</v>
+        <v>8.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>